<commit_message>
feat: add quotations workflow and UI polish; include updated app db
</commit_message>
<xml_diff>
--- a/JB10001_form_product.xlsx
+++ b/JB10001_form_product.xlsx
@@ -1023,7 +1023,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>01-03-2026 23:47:53</t>
+          <t>02-03-2026 02:02:56</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Thông tin</t>
+          <t>Item Size</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Lami: - | Size: 110*409 | PCS: 1 | UW: 0.063 | Qty: 4.499 | WT: 0.2834</t>
+          <t>110*409</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>50*50*50</t>
+          <t>2*2*2</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Lami: - | Size: 50 | PCS: 1 | UW: 23.15 | Qty: 50 | WT: 1157.5</t>
+          <t>50</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Lami: Yes | Size: 50*50 | PCS: 1 | UW: 0.2123 | Qty: 0.25 | WT: 0.0531</t>
+          <t>50*50</t>
         </is>
       </c>
     </row>

</xml_diff>